<commit_message>
feat: implement Strategy Pattern for Bipartite Matching, multi-domain retail knowledge base, and business presets
</commit_message>
<xml_diff>
--- a/sample-data/bao-cao-phan-phoi-fahasa.xlsx
+++ b/sample-data/bao-cao-phan-phoi-fahasa.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J11"/>
+  <dimension ref="A1:J5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -559,201 +559,9 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>5</v>
-      </c>
-      <c r="B6" t="str">
-        <v>9786045678904</v>
-      </c>
-      <c r="C6" t="str">
-        <v>Cà Phê Cùng Tony</v>
-      </c>
-      <c r="D6" t="str">
-        <v>CN00018</v>
-      </c>
-      <c r="E6" t="str">
-        <v>Nhà xuất bản Trẻ</v>
-      </c>
-      <c r="F6" t="str">
-        <v>95,000</v>
-      </c>
-      <c r="G6" t="str">
-        <v>2</v>
-      </c>
-      <c r="H6" t="str">
-        <v>1</v>
-      </c>
-      <c r="I6" t="str">
-        <v>1</v>
-      </c>
-      <c r="J6" t="str">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>6</v>
-      </c>
-      <c r="B7" t="str">
-        <v>9786045678905</v>
-      </c>
-      <c r="C7" t="str">
-        <v>Tôi Thấy Hoa Vàng Trên Cỏ Xanh</v>
-      </c>
-      <c r="D7" t="str">
-        <v>CN00018</v>
-      </c>
-      <c r="E7" t="str">
-        <v>Nhà xuất bản Trẻ</v>
-      </c>
-      <c r="F7" t="str">
-        <v>125,000</v>
-      </c>
-      <c r="G7" t="str">
-        <v>0</v>
-      </c>
-      <c r="H7" t="str">
-        <v>1</v>
-      </c>
-      <c r="I7" t="str">
-        <v>2</v>
-      </c>
-      <c r="J7" t="str">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>7</v>
-      </c>
-      <c r="B8" t="str">
-        <v>9786045678913</v>
-      </c>
-      <c r="C8" t="str">
-        <v>Dế Mèn Phiêu Lưu Ký (Ấn bản kỷ niệm)</v>
-      </c>
-      <c r="D8" t="str">
-        <v>CN00015</v>
-      </c>
-      <c r="E8" t="str">
-        <v>Chi nhánh Nhà xuất bản Kim Đồng tại Thành phố Hồ Chí Minh</v>
-      </c>
-      <c r="F8" t="str">
-        <v>55,000</v>
-      </c>
-      <c r="G8" t="str">
-        <v>5</v>
-      </c>
-      <c r="H8" t="str">
-        <v>3</v>
-      </c>
-      <c r="I8" t="str">
-        <v>4</v>
-      </c>
-      <c r="J8" t="str">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>8</v>
-      </c>
-      <c r="B9" t="str">
-        <v>9786045678910</v>
-      </c>
-      <c r="C9" t="str">
-        <v>Số Đỏ</v>
-      </c>
-      <c r="D9" t="str">
-        <v>CN00045</v>
-      </c>
-      <c r="E9" t="str">
-        <v>Nhà xuất bản Văn Học</v>
-      </c>
-      <c r="F9" t="str">
-        <v>65,000</v>
-      </c>
-      <c r="G9" t="str">
-        <v>1</v>
-      </c>
-      <c r="H9" t="str">
-        <v>0</v>
-      </c>
-      <c r="I9" t="str">
-        <v>1</v>
-      </c>
-      <c r="J9" t="str">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>9</v>
-      </c>
-      <c r="B10" t="str">
-        <v>9786045678911</v>
-      </c>
-      <c r="C10" t="str">
-        <v>Tư Duy Nhanh Và Chậm</v>
-      </c>
-      <c r="D10" t="str">
-        <v>CN00088</v>
-      </c>
-      <c r="E10" t="str">
-        <v>Nhà xuất bản Thế Giới</v>
-      </c>
-      <c r="F10" t="str">
-        <v>210,000</v>
-      </c>
-      <c r="G10" t="str">
-        <v>1</v>
-      </c>
-      <c r="H10" t="str">
-        <v>1</v>
-      </c>
-      <c r="I10" t="str">
-        <v>0</v>
-      </c>
-      <c r="J10" t="str">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v>10</v>
-      </c>
-      <c r="B11" t="str">
-        <v>9786045678918</v>
-      </c>
-      <c r="C11" t="str">
-        <v>Hạt Giống Tâm Hồn</v>
-      </c>
-      <c r="D11" t="str">
-        <v>CN00099</v>
-      </c>
-      <c r="E11" t="str">
-        <v>Nhà xuất bản Tổng Hợp TP.HCM</v>
-      </c>
-      <c r="F11" t="str">
-        <v>75,000</v>
-      </c>
-      <c r="G11" t="str">
-        <v>2</v>
-      </c>
-      <c r="H11" t="str">
-        <v>2</v>
-      </c>
-      <c r="I11" t="str">
-        <v>1</v>
-      </c>
-      <c r="J11" t="str">
-        <v>3</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J5"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: expand sample dataset to 5 files with 120 rows and rich error scenarios
</commit_message>
<xml_diff>
--- a/sample-data/bao-cao-phan-phoi-fahasa.xlsx
+++ b/sample-data/bao-cao-phan-phoi-fahasa.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="FAHASA Xuất Bán" sheetId="1" r:id="rId1"/>
+    <sheet name="FAHASA Xuất Bán Đa Chi Nhánh" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:K11"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -430,6 +430,9 @@
       <c r="J1" t="str">
         <v>GDNSTD - NS Thủ Đức</v>
       </c>
+      <c r="K1" t="str">
+        <v>GDNSPN - NS FAHASA Phú Nhuận</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -439,28 +442,31 @@
         <v>9786042392440</v>
       </c>
       <c r="C2" t="str">
-        <v>Mãi mãi tuổi hai mươi (Độc quyền - Bìa cứng)</v>
+        <v>Mãi Mãi Tuổi Hai Mươi (Độc Quyền - Bìa Cứng)</v>
       </c>
       <c r="D2" t="str">
         <v>CN00015</v>
       </c>
       <c r="E2" t="str">
-        <v>Chi nhánh Nhà xuất bản Kim Đồng tại Thành phố Hồ Chí Minh</v>
+        <v>Chi nhánh NXB Kim Đồng TP.HCM</v>
       </c>
       <c r="F2" t="str">
         <v>135,000</v>
       </c>
       <c r="G2" t="str">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H2" t="str">
         <v>1</v>
       </c>
       <c r="I2" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J2" t="str">
-        <v>2</v>
+        <v>5</v>
+      </c>
+      <c r="K2" t="str">
+        <v>4</v>
       </c>
     </row>
     <row r="3">
@@ -471,28 +477,31 @@
         <v>9786045678901</v>
       </c>
       <c r="C3" t="str">
-        <v>Đắc Nhân Tâm (Tái bản 2025)</v>
+        <v>Đắc Nhân Tâm (Tái Bản 2025)</v>
       </c>
       <c r="D3" t="str">
         <v>CN00018</v>
       </c>
       <c r="E3" t="str">
-        <v>Chi nhánh Công ty TNHH Văn Hóa Sáng Tạo Trí Việt</v>
+        <v>Chi nhánh Cty TNHH Văn Hóa Sáng Tạo Trí Việt</v>
       </c>
       <c r="F3" t="str">
         <v>86,000</v>
       </c>
       <c r="G3" t="str">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H3" t="str">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I3" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J3" t="str">
-        <v>4</v>
+        <v>8</v>
+      </c>
+      <c r="K3" t="str">
+        <v>6</v>
       </c>
     </row>
     <row r="4">
@@ -509,13 +518,13 @@
         <v>CN00022</v>
       </c>
       <c r="E4" t="str">
-        <v>Công ty Cổ phần Văn hóa &amp; Truyền thông Nhã Nam</v>
+        <v>Cty CP Văn hóa &amp; Truyền thông Nhã Nam</v>
       </c>
       <c r="F4" t="str">
         <v>79,000</v>
       </c>
       <c r="G4" t="str">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H4" t="str">
         <v>0</v>
@@ -524,6 +533,9 @@
         <v>3</v>
       </c>
       <c r="J4" t="str">
+        <v>7</v>
+      </c>
+      <c r="K4" t="str">
         <v>5</v>
       </c>
     </row>
@@ -541,13 +553,13 @@
         <v>CN00030</v>
       </c>
       <c r="E5" t="str">
-        <v>Nhà xuất bản Hội Nhà Văn</v>
+        <v>NXB Hội Nhà Văn</v>
       </c>
       <c r="F5" t="str">
         <v>90,000</v>
       </c>
       <c r="G5" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H5" t="str">
         <v>2</v>
@@ -556,12 +568,225 @@
         <v>0</v>
       </c>
       <c r="J5" t="str">
-        <v>3</v>
+        <v>4</v>
+      </c>
+      <c r="K5" t="str">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>5</v>
+      </c>
+      <c r="B6" t="str">
+        <v>9786045678904</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Cà Phê Cùng Tony</v>
+      </c>
+      <c r="D6" t="str">
+        <v>CN00018</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Chi nhánh Cty TNHH Văn Hóa Sáng Tạo Trí Việt</v>
+      </c>
+      <c r="F6" t="str">
+        <v>72,000</v>
+      </c>
+      <c r="G6" t="str">
+        <v>3</v>
+      </c>
+      <c r="H6" t="str">
+        <v>1</v>
+      </c>
+      <c r="I6" t="str">
+        <v>1</v>
+      </c>
+      <c r="J6" t="str">
+        <v>5</v>
+      </c>
+      <c r="K6" t="str">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>6</v>
+      </c>
+      <c r="B7" t="str">
+        <v>9786045678905</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Tôi Thấy Hoa Vàng Trên Cỏ Xanh</v>
+      </c>
+      <c r="D7" t="str">
+        <v>CN00018</v>
+      </c>
+      <c r="E7" t="str">
+        <v>Chi nhánh Cty TNHH Văn Hóa Sáng Tạo Trí Việt</v>
+      </c>
+      <c r="F7" t="str">
+        <v>85,000</v>
+      </c>
+      <c r="G7" t="str">
+        <v>2</v>
+      </c>
+      <c r="H7" t="str">
+        <v>1</v>
+      </c>
+      <c r="I7" t="str">
+        <v>2</v>
+      </c>
+      <c r="J7" t="str">
+        <v>3</v>
+      </c>
+      <c r="K7" t="str">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>7</v>
+      </c>
+      <c r="B8" t="str">
+        <v>9786045678906</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Cho Tôi Xin Một Vé Đi Tuổi Thơ</v>
+      </c>
+      <c r="D8" t="str">
+        <v>CN00018</v>
+      </c>
+      <c r="E8" t="str">
+        <v>Chi nhánh Cty TNHH Văn Hóa Sáng Tạo Trí Việt</v>
+      </c>
+      <c r="F8" t="str">
+        <v>65,000</v>
+      </c>
+      <c r="G8" t="str">
+        <v>1</v>
+      </c>
+      <c r="H8" t="str">
+        <v>0</v>
+      </c>
+      <c r="I8" t="str">
+        <v>1</v>
+      </c>
+      <c r="J8" t="str">
+        <v>2</v>
+      </c>
+      <c r="K8" t="str">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>8</v>
+      </c>
+      <c r="B9" t="str">
+        <v>9786045678907</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Sapiens: Lược Sử Loài Người</v>
+      </c>
+      <c r="D9" t="str">
+        <v>CN00040</v>
+      </c>
+      <c r="E9" t="str">
+        <v>NXB Thế Giới</v>
+      </c>
+      <c r="F9" t="str">
+        <v>189,000</v>
+      </c>
+      <c r="G9" t="str">
+        <v>1</v>
+      </c>
+      <c r="H9" t="str">
+        <v>1</v>
+      </c>
+      <c r="I9" t="str">
+        <v>0</v>
+      </c>
+      <c r="J9" t="str">
+        <v>2</v>
+      </c>
+      <c r="K9" t="str">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>9</v>
+      </c>
+      <c r="B10" t="str">
+        <v>9786045678908</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Atomic Habits - Thay Đổi Tí Hon Hiệu Quả Bất Ngờ</v>
+      </c>
+      <c r="D10" t="str">
+        <v>CN00040</v>
+      </c>
+      <c r="E10" t="str">
+        <v>NXB Thế Giới</v>
+      </c>
+      <c r="F10" t="str">
+        <v>149,000</v>
+      </c>
+      <c r="G10" t="str">
+        <v>2</v>
+      </c>
+      <c r="H10" t="str">
+        <v>0</v>
+      </c>
+      <c r="I10" t="str">
+        <v>1</v>
+      </c>
+      <c r="J10" t="str">
+        <v>3</v>
+      </c>
+      <c r="K10" t="str">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>10</v>
+      </c>
+      <c r="B11" t="str">
+        <v>9786045678909</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Dám Bị Ghét</v>
+      </c>
+      <c r="D11" t="str">
+        <v>CN00035</v>
+      </c>
+      <c r="E11" t="str">
+        <v>NXB Lao Động</v>
+      </c>
+      <c r="F11" t="str">
+        <v>115,000</v>
+      </c>
+      <c r="G11" t="str">
+        <v>1</v>
+      </c>
+      <c r="H11" t="str">
+        <v>1</v>
+      </c>
+      <c r="I11" t="str">
+        <v>0</v>
+      </c>
+      <c r="J11" t="str">
+        <v>2</v>
+      </c>
+      <c r="K11" t="str">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K11"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix: auto-detect English/underscored headers, fix ISBN prefix filter and valid checksums in sample data
</commit_message>
<xml_diff>
--- a/sample-data/bao-cao-phan-phoi-fahasa.xlsx
+++ b/sample-data/bao-cao-phan-phoi-fahasa.xlsx
@@ -474,7 +474,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="str">
-        <v>9786045678901</v>
+        <v>9786045678909</v>
       </c>
       <c r="C3" t="str">
         <v>Đắc Nhân Tâm (Tái Bản 2025)</v>
@@ -509,7 +509,7 @@
         <v>3</v>
       </c>
       <c r="B4" t="str">
-        <v>9786045678902</v>
+        <v>9786045678916</v>
       </c>
       <c r="C4" t="str">
         <v>Nhà Giả Kim</v>
@@ -544,7 +544,7 @@
         <v>4</v>
       </c>
       <c r="B5" t="str">
-        <v>9786045678903</v>
+        <v>9786045678923</v>
       </c>
       <c r="C5" t="str">
         <v>Tuổi Trẻ Đáng Giá Bao Nhiêu</v>
@@ -579,7 +579,7 @@
         <v>5</v>
       </c>
       <c r="B6" t="str">
-        <v>9786045678904</v>
+        <v>9786045678930</v>
       </c>
       <c r="C6" t="str">
         <v>Cà Phê Cùng Tony</v>
@@ -614,7 +614,7 @@
         <v>6</v>
       </c>
       <c r="B7" t="str">
-        <v>9786045678905</v>
+        <v>9786045678947</v>
       </c>
       <c r="C7" t="str">
         <v>Tôi Thấy Hoa Vàng Trên Cỏ Xanh</v>
@@ -649,7 +649,7 @@
         <v>7</v>
       </c>
       <c r="B8" t="str">
-        <v>9786045678906</v>
+        <v>9786045678954</v>
       </c>
       <c r="C8" t="str">
         <v>Cho Tôi Xin Một Vé Đi Tuổi Thơ</v>
@@ -684,7 +684,7 @@
         <v>8</v>
       </c>
       <c r="B9" t="str">
-        <v>9786045678907</v>
+        <v>9786045678961</v>
       </c>
       <c r="C9" t="str">
         <v>Sapiens: Lược Sử Loài Người</v>
@@ -719,7 +719,7 @@
         <v>9</v>
       </c>
       <c r="B10" t="str">
-        <v>9786045678908</v>
+        <v>9786045678978</v>
       </c>
       <c r="C10" t="str">
         <v>Atomic Habits - Thay Đổi Tí Hon Hiệu Quả Bất Ngờ</v>
@@ -754,7 +754,7 @@
         <v>10</v>
       </c>
       <c r="B11" t="str">
-        <v>9786045678909</v>
+        <v>9786045678985</v>
       </c>
       <c r="C11" t="str">
         <v>Dám Bị Ghét</v>

</xml_diff>